<commit_message>
feat(pro): 易贡 BH02 案例标定 bed=0.05/200s，并补写 t=0 初始帧
数据（suanfa/Pro/task1 的 p.txt 与 参数表.xlsx）：bed 由 0.2 降为 0.05 rad（约 2.9° 有效基底摩擦角）、输出间距 10 s、计算时长 200 s。BH02 物源紧邻堰塞湖、最陡路径仅约 226 m、落差约 34 m，基底摩擦角是运动速度主控参数：0.2 rad 时前 40 s 质心只移动约 40 m，0.05 rad 时 t=20 s 已有约 54% 体积入湖、t=200 s 约 95%。

脚本（run_pro.py）：数值内核只在跨越输出间隔时回调、从不给出 t=0 状态，导致动画从第一个输出时刻开始、缺少完好物源初始态；现在统一补写一帧初始场。
</commit_message>
<xml_diff>
--- a/suanfa/Pro/task1/参数表.xlsx
+++ b/suanfa/Pro/task1/参数表.xlsx
@@ -1,106 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <workbookPr/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="122211"/>
+  <definedNames/>
+  <calcPr calcId="122211" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
-  <si>
-    <t>参数</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>取值</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>基底摩擦角 bed</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>网格长度   dx</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>网格宽度   dy</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>计算时间   Tmax</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>100s</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>24°</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>曼宁摩擦系数 nn</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>滑坡密度  rous</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>2700 kg/m3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>河水密度 rouf</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1000 kg/m3</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>输出间距 Interval</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>20m</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <family val="3"/>
       <sz val="9"/>
-      <name val="宋体"/>
-      <family val="3"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -119,21 +55,83 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -423,109 +421,162 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B9"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="27" customWidth="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1.2500000000000001E-2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>9</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>参数</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>取值</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>基底摩擦角 bed</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>0.05（约 2.9°，有效基底摩擦角）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>曼宁摩擦系数 nn</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>0.0125</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>网格长度   dx</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>20m</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>网格宽度   dy</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>20m</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>滑坡密度  rous</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2700 kg/m3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>河水密度 rouf</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1000 kg/m3</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>输出间距 Interval</t>
+        </is>
+      </c>
+      <c r="B8" s="1" t="n">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="1">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>计算时间   Tmax</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>200s</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>标定说明</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>易贡 BH02 案例标定：物源紧邻堰塞湖、天然落差约 34 m，基底摩擦角为运动速度主控参数；取 0.05 rad（约 2.9°）时 t=20 s 入湖约 54%、t=40 s 约 79%、t=200 s 约 95%</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup orientation="portrait" paperSize="9"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData/>
-  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>